<commit_message>
Updated date on 7
</commit_message>
<xml_diff>
--- a/assets_output/07_multinomial_logistic_regression.xlsx
+++ b/assets_output/07_multinomial_logistic_regression.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1289" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1289" uniqueCount="186">
   <si>
     <t>MNLogit: 'Entry point into BAHSA services (pathway type and level)', table 0</t>
   </si>
@@ -49,7 +49,7 @@
     <t>y</t>
   </si>
   <si>
-    <t>2026-05-17 15:54</t>
+    <t>2026-05-18 18:16</t>
   </si>
   <si>
     <t>4355</t>
@@ -449,6 +449,9 @@
   </si>
   <si>
     <t>after_rt_ret_within_2y</t>
+  </si>
+  <si>
+    <t>2026-05-18 18:17</t>
   </si>
   <si>
     <t>730</t>
@@ -9897,7 +9900,7 @@
         <v>18</v>
       </c>
       <c r="E451" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="452" spans="1:7">
@@ -9908,13 +9911,13 @@
         <v>3</v>
       </c>
       <c r="C452" t="s">
-        <v>11</v>
+        <v>145</v>
       </c>
       <c r="D452" t="s">
         <v>19</v>
       </c>
       <c r="E452" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="453" spans="1:7">
@@ -9925,13 +9928,13 @@
         <v>4</v>
       </c>
       <c r="C453" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D453" t="s">
         <v>20</v>
       </c>
       <c r="E453" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="454" spans="1:7">
@@ -9942,13 +9945,13 @@
         <v>5</v>
       </c>
       <c r="C454" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D454" t="s">
         <v>21</v>
       </c>
       <c r="E454" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="455" spans="1:7">
@@ -9959,13 +9962,13 @@
         <v>6</v>
       </c>
       <c r="C455" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D455" t="s">
         <v>22</v>
       </c>
       <c r="E455" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="456" spans="1:7">
@@ -9982,7 +9985,7 @@
         <v>23</v>
       </c>
       <c r="E456" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="457" spans="1:7">
@@ -10004,7 +10007,7 @@
     </row>
     <row r="459" spans="1:7">
       <c r="A459" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="460" spans="1:7">
@@ -10052,7 +10055,7 @@
     </row>
     <row r="462" spans="1:7">
       <c r="A462" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B462">
         <v>2.5</v>
@@ -10121,7 +10124,7 @@
     </row>
     <row r="466" spans="1:6">
       <c r="A466" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="467" spans="1:6">
@@ -10163,7 +10166,7 @@
     </row>
     <row r="469" spans="1:6">
       <c r="A469" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B469">
         <v>0</v>
@@ -10223,7 +10226,7 @@
     </row>
     <row r="473" spans="1:6">
       <c r="A473" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="474" spans="1:6">
@@ -10265,13 +10268,13 @@
         <v>2</v>
       </c>
       <c r="C476" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D476" t="s">
         <v>18</v>
       </c>
       <c r="E476" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="477" spans="1:6">
@@ -10282,13 +10285,13 @@
         <v>3</v>
       </c>
       <c r="C477" t="s">
-        <v>11</v>
+        <v>145</v>
       </c>
       <c r="D477" t="s">
         <v>19</v>
       </c>
       <c r="E477" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="478" spans="1:6">
@@ -10299,13 +10302,13 @@
         <v>4</v>
       </c>
       <c r="C478" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D478" t="s">
         <v>20</v>
       </c>
       <c r="E478" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="479" spans="1:6">
@@ -10316,13 +10319,13 @@
         <v>5</v>
       </c>
       <c r="C479" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D479" t="s">
         <v>21</v>
       </c>
       <c r="E479" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="480" spans="1:6">
@@ -10333,13 +10336,13 @@
         <v>6</v>
       </c>
       <c r="C480" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D480" t="s">
         <v>22</v>
       </c>
       <c r="E480" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="481" spans="1:8">
@@ -10356,7 +10359,7 @@
         <v>23</v>
       </c>
       <c r="E481" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="482" spans="1:8">
@@ -10378,12 +10381,12 @@
     </row>
     <row r="484" spans="1:8">
       <c r="A484" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="485" spans="1:8">
       <c r="B485" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C485" s="1" t="s">
         <v>34</v>
@@ -10718,12 +10721,12 @@
     </row>
     <row r="499" spans="1:8">
       <c r="A499" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="500" spans="1:8">
       <c r="B500" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C500" s="1" t="s">
         <v>34</v>
@@ -11058,12 +11061,12 @@
     </row>
     <row r="514" spans="1:8">
       <c r="A514" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="515" spans="1:8">
       <c r="B515" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C515" s="1" t="s">
         <v>34</v>
@@ -11398,12 +11401,12 @@
     </row>
     <row r="529" spans="1:8">
       <c r="A529" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="530" spans="1:8">
       <c r="B530" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C530" s="1" t="s">
         <v>34</v>
@@ -11738,12 +11741,12 @@
     </row>
     <row r="544" spans="1:8">
       <c r="A544" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="545" spans="1:8">
       <c r="B545" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C545" s="1" t="s">
         <v>34</v>
@@ -12078,12 +12081,12 @@
     </row>
     <row r="559" spans="1:8">
       <c r="A559" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="560" spans="1:8">
       <c r="B560" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C560" s="1" t="s">
         <v>34</v>
@@ -12418,7 +12421,7 @@
     </row>
     <row r="574" spans="1:8">
       <c r="A574" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="575" spans="1:8">
@@ -12673,7 +12676,7 @@
     </row>
     <row r="588" spans="1:7">
       <c r="A588" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B588" s="1" t="s">
         <v>40</v>
@@ -12906,7 +12909,7 @@
     </row>
     <row r="600" spans="1:7">
       <c r="A600" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B600" s="1" t="s">
         <v>40</v>
@@ -13139,7 +13142,7 @@
     </row>
     <row r="612" spans="1:7">
       <c r="A612" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B612" s="1" t="s">
         <v>40</v>
@@ -13363,7 +13366,7 @@
     </row>
     <row r="624" spans="1:7">
       <c r="A624" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B624" s="1" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
Updated scales and presentation of visualisations
</commit_message>
<xml_diff>
--- a/assets_output/07_multinomial_logistic_regression.xlsx
+++ b/assets_output/07_multinomial_logistic_regression.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1279" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1279" uniqueCount="186">
   <si>
     <t>MNLogit: 'Entry point into BAHSA services (pathway type and level)', table 0</t>
   </si>
@@ -49,7 +49,7 @@
     <t>y</t>
   </si>
   <si>
-    <t>2026-05-22 14:15</t>
+    <t>2026-05-22 18:13</t>
   </si>
   <si>
     <t>3391</t>
@@ -371,6 +371,9 @@
   </si>
   <si>
     <t>multiple_returns</t>
+  </si>
+  <si>
+    <t>2026-05-22 18:14</t>
   </si>
   <si>
     <t>6</t>
@@ -8870,7 +8873,7 @@
         <v>18</v>
       </c>
       <c r="E389" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="390" spans="1:7">
@@ -8881,13 +8884,13 @@
         <v>3</v>
       </c>
       <c r="C390" t="s">
-        <v>11</v>
+        <v>119</v>
       </c>
       <c r="D390" t="s">
         <v>19</v>
       </c>
       <c r="E390" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="391" spans="1:7">
@@ -8904,7 +8907,7 @@
         <v>20</v>
       </c>
       <c r="E391" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="392" spans="1:7">
@@ -8915,13 +8918,13 @@
         <v>5</v>
       </c>
       <c r="C392" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D392" t="s">
         <v>21</v>
       </c>
       <c r="E392" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="393" spans="1:7">
@@ -8932,13 +8935,13 @@
         <v>6</v>
       </c>
       <c r="C393" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D393" t="s">
         <v>22</v>
       </c>
       <c r="E393" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="394" spans="1:7">
@@ -8955,7 +8958,7 @@
         <v>23</v>
       </c>
       <c r="E394" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="395" spans="1:7">
@@ -8966,7 +8969,7 @@
         <v>8</v>
       </c>
       <c r="C395" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D395" t="s">
         <v>24</v>
@@ -8977,7 +8980,7 @@
     </row>
     <row r="397" spans="1:7">
       <c r="A397" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="398" spans="1:7">
@@ -8988,10 +8991,10 @@
         <v>35</v>
       </c>
       <c r="D398" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E398" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F398" s="1" t="s">
         <v>38</v>
@@ -9163,7 +9166,7 @@
     </row>
     <row r="407" spans="1:7">
       <c r="A407" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="408" spans="1:7">
@@ -9330,7 +9333,7 @@
     </row>
     <row r="418" spans="1:7">
       <c r="A418" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="419" spans="1:7">
@@ -9372,13 +9375,13 @@
         <v>2</v>
       </c>
       <c r="C421" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D421" t="s">
         <v>18</v>
       </c>
       <c r="E421" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="422" spans="1:7">
@@ -9389,13 +9392,13 @@
         <v>3</v>
       </c>
       <c r="C422" t="s">
-        <v>11</v>
+        <v>119</v>
       </c>
       <c r="D422" t="s">
         <v>19</v>
       </c>
       <c r="E422" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="423" spans="1:7">
@@ -9412,7 +9415,7 @@
         <v>20</v>
       </c>
       <c r="E423" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="424" spans="1:7">
@@ -9423,13 +9426,13 @@
         <v>5</v>
       </c>
       <c r="C424" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D424" t="s">
         <v>21</v>
       </c>
       <c r="E424" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="425" spans="1:7">
@@ -9440,13 +9443,13 @@
         <v>6</v>
       </c>
       <c r="C425" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D425" t="s">
         <v>22</v>
       </c>
       <c r="E425" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="426" spans="1:7">
@@ -9463,7 +9466,7 @@
         <v>23</v>
       </c>
       <c r="E426" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="427" spans="1:7">
@@ -9474,7 +9477,7 @@
         <v>8</v>
       </c>
       <c r="C427" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D427" t="s">
         <v>24</v>
@@ -9485,7 +9488,7 @@
     </row>
     <row r="429" spans="1:7">
       <c r="A429" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="430" spans="1:7">
@@ -9496,10 +9499,10 @@
         <v>35</v>
       </c>
       <c r="D430" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E430" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F430" s="1" t="s">
         <v>38</v>
@@ -9671,7 +9674,7 @@
     </row>
     <row r="439" spans="1:7">
       <c r="A439" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="440" spans="1:7">
@@ -9838,7 +9841,7 @@
     </row>
     <row r="450" spans="1:7">
       <c r="A450" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="451" spans="1:7">
@@ -9880,13 +9883,13 @@
         <v>2</v>
       </c>
       <c r="C453" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="D453" t="s">
         <v>18</v>
       </c>
       <c r="E453" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="454" spans="1:7">
@@ -9897,13 +9900,13 @@
         <v>3</v>
       </c>
       <c r="C454" t="s">
-        <v>11</v>
+        <v>119</v>
       </c>
       <c r="D454" t="s">
         <v>19</v>
       </c>
       <c r="E454" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="455" spans="1:7">
@@ -9914,13 +9917,13 @@
         <v>4</v>
       </c>
       <c r="C455" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D455" t="s">
         <v>20</v>
       </c>
       <c r="E455" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="456" spans="1:7">
@@ -9931,13 +9934,13 @@
         <v>5</v>
       </c>
       <c r="C456" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D456" t="s">
         <v>21</v>
       </c>
       <c r="E456" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="457" spans="1:7">
@@ -9948,13 +9951,13 @@
         <v>6</v>
       </c>
       <c r="C457" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D457" t="s">
         <v>22</v>
       </c>
       <c r="E457" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="458" spans="1:7">
@@ -9971,7 +9974,7 @@
         <v>23</v>
       </c>
       <c r="E458" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="459" spans="1:7">
@@ -9993,7 +9996,7 @@
     </row>
     <row r="461" spans="1:7">
       <c r="A461" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="462" spans="1:7">
@@ -10004,10 +10007,10 @@
         <v>35</v>
       </c>
       <c r="D462" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E462" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F462" s="1" t="s">
         <v>38</v>
@@ -10041,7 +10044,7 @@
     </row>
     <row r="464" spans="1:7">
       <c r="A464" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B464">
         <v>2.4</v>
@@ -10110,7 +10113,7 @@
     </row>
     <row r="468" spans="1:7">
       <c r="A468" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="469" spans="1:7">
@@ -10152,7 +10155,7 @@
     </row>
     <row r="471" spans="1:7">
       <c r="A471" s="1" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B471">
         <v>0</v>
@@ -10214,7 +10217,7 @@
     </row>
     <row r="476" spans="1:7">
       <c r="A476" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="477" spans="1:7">
@@ -10256,13 +10259,13 @@
         <v>2</v>
       </c>
       <c r="C479" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D479" t="s">
         <v>18</v>
       </c>
       <c r="E479" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="480" spans="1:7">
@@ -10273,13 +10276,13 @@
         <v>3</v>
       </c>
       <c r="C480" t="s">
-        <v>11</v>
+        <v>119</v>
       </c>
       <c r="D480" t="s">
         <v>19</v>
       </c>
       <c r="E480" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="481" spans="1:8">
@@ -10290,13 +10293,13 @@
         <v>4</v>
       </c>
       <c r="C481" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D481" t="s">
         <v>20</v>
       </c>
       <c r="E481" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="482" spans="1:8">
@@ -10307,13 +10310,13 @@
         <v>5</v>
       </c>
       <c r="C482" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D482" t="s">
         <v>21</v>
       </c>
       <c r="E482" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="483" spans="1:8">
@@ -10324,13 +10327,13 @@
         <v>6</v>
       </c>
       <c r="C483" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D483" t="s">
         <v>22</v>
       </c>
       <c r="E483" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="484" spans="1:8">
@@ -10347,7 +10350,7 @@
         <v>23</v>
       </c>
       <c r="E484" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="485" spans="1:8">
@@ -10369,12 +10372,12 @@
     </row>
     <row r="487" spans="1:8">
       <c r="A487" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="488" spans="1:8">
       <c r="B488" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C488" s="1" t="s">
         <v>34</v>
@@ -10709,12 +10712,12 @@
     </row>
     <row r="502" spans="1:8">
       <c r="A502" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="503" spans="1:8">
       <c r="B503" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C503" s="1" t="s">
         <v>34</v>
@@ -11049,12 +11052,12 @@
     </row>
     <row r="517" spans="1:8">
       <c r="A517" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="518" spans="1:8">
       <c r="B518" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C518" s="1" t="s">
         <v>34</v>
@@ -11389,12 +11392,12 @@
     </row>
     <row r="532" spans="1:8">
       <c r="A532" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="533" spans="1:8">
       <c r="B533" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C533" s="1" t="s">
         <v>34</v>
@@ -11729,12 +11732,12 @@
     </row>
     <row r="547" spans="1:8">
       <c r="A547" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="548" spans="1:8">
       <c r="B548" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C548" s="1" t="s">
         <v>34</v>
@@ -12069,12 +12072,12 @@
     </row>
     <row r="562" spans="1:8">
       <c r="A562" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="563" spans="1:8">
       <c r="B563" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C563" s="1" t="s">
         <v>34</v>
@@ -12409,7 +12412,7 @@
     </row>
     <row r="577" spans="1:7">
       <c r="A577" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="578" spans="1:7">
@@ -12661,7 +12664,7 @@
     </row>
     <row r="591" spans="1:7">
       <c r="A591" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B591" s="1" t="s">
         <v>40</v>
@@ -12888,7 +12891,7 @@
     </row>
     <row r="603" spans="1:7">
       <c r="A603" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B603" s="1" t="s">
         <v>40</v>
@@ -13118,7 +13121,7 @@
     </row>
     <row r="615" spans="1:7">
       <c r="A615" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B615" s="1" t="s">
         <v>40</v>
@@ -13342,7 +13345,7 @@
     </row>
     <row r="627" spans="1:7">
       <c r="A627" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B627" s="1" t="s">
         <v>40</v>

</xml_diff>

<commit_message>
Added private rented affordability figure
</commit_message>
<xml_diff>
--- a/assets_output/07_multinomial_logistic_regression.xlsx
+++ b/assets_output/07_multinomial_logistic_regression.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1261" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1261" uniqueCount="185">
   <si>
     <t>MNLogit: 'Entry point into BAHSA services (pathway type and level)', table 0</t>
   </si>
@@ -49,7 +49,7 @@
     <t>y</t>
   </si>
   <si>
-    <t>2026-05-31 10:30</t>
+    <t>2026-05-31 11:22</t>
   </si>
   <si>
     <t>3391</t>
@@ -245,9 +245,6 @@
   </si>
   <si>
     <t>rt_outcome</t>
-  </si>
-  <si>
-    <t>2026-05-31 10:31</t>
   </si>
   <si>
     <t>2195</t>
@@ -5374,7 +5371,7 @@
         <v>18</v>
       </c>
       <c r="E213" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="214" spans="1:8">
@@ -5385,13 +5382,13 @@
         <v>3</v>
       </c>
       <c r="C214" t="s">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="D214" t="s">
         <v>19</v>
       </c>
       <c r="E214" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="215" spans="1:8">
@@ -5402,13 +5399,13 @@
         <v>4</v>
       </c>
       <c r="C215" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D215" t="s">
         <v>20</v>
       </c>
       <c r="E215" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="216" spans="1:8">
@@ -5419,13 +5416,13 @@
         <v>5</v>
       </c>
       <c r="C216" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D216" t="s">
         <v>21</v>
       </c>
       <c r="E216" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="217" spans="1:8">
@@ -5436,13 +5433,13 @@
         <v>6</v>
       </c>
       <c r="C217" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D217" t="s">
         <v>22</v>
       </c>
       <c r="E217" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="218" spans="1:8">
@@ -5459,7 +5456,7 @@
         <v>23</v>
       </c>
       <c r="E218" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="219" spans="1:8">
@@ -5470,7 +5467,7 @@
         <v>8</v>
       </c>
       <c r="C219" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D219" t="s">
         <v>24</v>
@@ -5481,12 +5478,12 @@
     </row>
     <row r="221" spans="1:8">
       <c r="A221" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="222" spans="1:8">
       <c r="B222" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C222" s="1" t="s">
         <v>34</v>
@@ -5613,10 +5610,10 @@
     </row>
     <row r="227" spans="1:8">
       <c r="A227" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B227" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C227">
         <v>0.3</v>
@@ -5743,10 +5740,10 @@
     </row>
     <row r="232" spans="1:8">
       <c r="A232" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B232" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C232">
         <v>1.7</v>
@@ -5795,12 +5792,12 @@
     </row>
     <row r="235" spans="1:8">
       <c r="A235" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="236" spans="1:8">
       <c r="B236" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C236" s="1" t="s">
         <v>34</v>
@@ -5927,10 +5924,10 @@
     </row>
     <row r="241" spans="1:8">
       <c r="A241" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B241" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C241">
         <v>0.1</v>
@@ -6057,10 +6054,10 @@
     </row>
     <row r="246" spans="1:8">
       <c r="A246" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B246" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C246">
         <v>2</v>
@@ -6109,12 +6106,12 @@
     </row>
     <row r="249" spans="1:8">
       <c r="A249" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="250" spans="1:8">
       <c r="B250" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C250" s="1" t="s">
         <v>34</v>
@@ -6241,10 +6238,10 @@
     </row>
     <row r="255" spans="1:8">
       <c r="A255" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B255" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C255">
         <v>-0.5</v>
@@ -6371,10 +6368,10 @@
     </row>
     <row r="260" spans="1:8">
       <c r="A260" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B260" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C260">
         <v>2.9</v>
@@ -6423,7 +6420,7 @@
     </row>
     <row r="263" spans="1:8">
       <c r="A263" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="264" spans="1:8">
@@ -6445,7 +6442,7 @@
     </row>
     <row r="265" spans="1:8">
       <c r="A265" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B265" s="1" t="s">
         <v>40</v>
@@ -6469,7 +6466,7 @@
     <row r="266" spans="1:8">
       <c r="A266" s="1"/>
       <c r="B266" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C266">
         <v>0.3</v>
@@ -6577,7 +6574,7 @@
     <row r="272" spans="1:8">
       <c r="A272" s="1"/>
       <c r="B272" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C272">
         <v>0</v>
@@ -6654,7 +6651,7 @@
     </row>
     <row r="276" spans="1:7">
       <c r="A276" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B276" s="1" t="s">
         <v>40</v>
@@ -6678,7 +6675,7 @@
     <row r="277" spans="1:7">
       <c r="A277" s="1"/>
       <c r="B277" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C277">
         <v>0</v>
@@ -6801,7 +6798,7 @@
     <row r="283" spans="1:7">
       <c r="A283" s="1"/>
       <c r="B283" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C283">
         <v>0</v>
@@ -6881,7 +6878,7 @@
     </row>
     <row r="287" spans="1:7">
       <c r="A287" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B287" s="1" t="s">
         <v>40</v>
@@ -6905,7 +6902,7 @@
     <row r="288" spans="1:7">
       <c r="A288" s="1"/>
       <c r="B288" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C288">
         <v>0.3</v>
@@ -7022,7 +7019,7 @@
     <row r="294" spans="1:7">
       <c r="A294" s="1"/>
       <c r="B294" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C294">
         <v>0</v>
@@ -7102,7 +7099,7 @@
     </row>
     <row r="299" spans="1:7">
       <c r="A299" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="300" spans="1:7">
@@ -7144,13 +7141,13 @@
         <v>2</v>
       </c>
       <c r="C302" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D302" t="s">
         <v>18</v>
       </c>
       <c r="E302" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="303" spans="1:7">
@@ -7161,13 +7158,13 @@
         <v>3</v>
       </c>
       <c r="C303" t="s">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="D303" t="s">
         <v>19</v>
       </c>
       <c r="E303" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="304" spans="1:7">
@@ -7178,13 +7175,13 @@
         <v>4</v>
       </c>
       <c r="C304" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D304" t="s">
         <v>20</v>
       </c>
       <c r="E304" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="305" spans="1:8">
@@ -7195,13 +7192,13 @@
         <v>5</v>
       </c>
       <c r="C305" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D305" t="s">
         <v>21</v>
       </c>
       <c r="E305" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="306" spans="1:8">
@@ -7212,13 +7209,13 @@
         <v>6</v>
       </c>
       <c r="C306" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D306" t="s">
         <v>22</v>
       </c>
       <c r="E306" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="307" spans="1:8">
@@ -7235,7 +7232,7 @@
         <v>23</v>
       </c>
       <c r="E307" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="308" spans="1:8">
@@ -7246,7 +7243,7 @@
         <v>8</v>
       </c>
       <c r="C308" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D308" t="s">
         <v>24</v>
@@ -7257,12 +7254,12 @@
     </row>
     <row r="310" spans="1:8">
       <c r="A310" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="311" spans="1:8">
       <c r="B311" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C311" s="1" t="s">
         <v>34</v>
@@ -7363,10 +7360,10 @@
     </row>
     <row r="315" spans="1:8">
       <c r="A315" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B315" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C315">
         <v>0.3</v>
@@ -7493,10 +7490,10 @@
     </row>
     <row r="320" spans="1:8">
       <c r="A320" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B320" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C320">
         <v>1.7</v>
@@ -7519,12 +7516,12 @@
     </row>
     <row r="322" spans="1:8">
       <c r="A322" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="323" spans="1:8">
       <c r="B323" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C323" s="1" t="s">
         <v>34</v>
@@ -7625,10 +7622,10 @@
     </row>
     <row r="327" spans="1:8">
       <c r="A327" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B327" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C327">
         <v>0.2</v>
@@ -7755,10 +7752,10 @@
     </row>
     <row r="332" spans="1:8">
       <c r="A332" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B332" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C332">
         <v>1.8</v>
@@ -7781,12 +7778,12 @@
     </row>
     <row r="334" spans="1:8">
       <c r="A334" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="335" spans="1:8">
       <c r="B335" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C335" s="1" t="s">
         <v>34</v>
@@ -7887,10 +7884,10 @@
     </row>
     <row r="339" spans="1:8">
       <c r="A339" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B339" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C339">
         <v>-0.5</v>
@@ -8017,10 +8014,10 @@
     </row>
     <row r="344" spans="1:8">
       <c r="A344" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B344" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C344">
         <v>2.2</v>
@@ -8043,7 +8040,7 @@
     </row>
     <row r="346" spans="1:8">
       <c r="A346" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="347" spans="1:8">
@@ -8065,7 +8062,7 @@
     </row>
     <row r="348" spans="1:8">
       <c r="A348" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B348" s="1" t="s">
         <v>40</v>
@@ -8089,7 +8086,7 @@
     <row r="349" spans="1:8">
       <c r="A349" s="1"/>
       <c r="B349" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C349">
         <v>0.3</v>
@@ -8161,7 +8158,7 @@
     <row r="353" spans="1:7">
       <c r="A353" s="1"/>
       <c r="B353" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C353">
         <v>0.1</v>
@@ -8235,7 +8232,7 @@
     </row>
     <row r="357" spans="1:7">
       <c r="A357" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B357" s="1" t="s">
         <v>40</v>
@@ -8259,7 +8256,7 @@
     <row r="358" spans="1:7">
       <c r="A358" s="1"/>
       <c r="B358" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C358">
         <v>0</v>
@@ -8343,7 +8340,7 @@
     <row r="362" spans="1:7">
       <c r="A362" s="1"/>
       <c r="B362" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C362">
         <v>0</v>
@@ -8423,7 +8420,7 @@
     </row>
     <row r="366" spans="1:7">
       <c r="A366" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B366" s="1" t="s">
         <v>40</v>
@@ -8447,7 +8444,7 @@
     <row r="367" spans="1:7">
       <c r="A367" s="1"/>
       <c r="B367" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C367">
         <v>0.1</v>
@@ -8525,7 +8522,7 @@
     <row r="371" spans="1:7">
       <c r="A371" s="1"/>
       <c r="B371" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C371">
         <v>0</v>
@@ -8605,7 +8602,7 @@
     </row>
     <row r="376" spans="1:7">
       <c r="A376" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="377" spans="1:7">
@@ -8630,7 +8627,7 @@
         <v>1</v>
       </c>
       <c r="C378" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D378" t="s">
         <v>17</v>
@@ -8647,13 +8644,13 @@
         <v>2</v>
       </c>
       <c r="C379" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D379" t="s">
         <v>18</v>
       </c>
       <c r="E379" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="380" spans="1:7">
@@ -8664,13 +8661,13 @@
         <v>3</v>
       </c>
       <c r="C380" t="s">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="D380" t="s">
         <v>19</v>
       </c>
       <c r="E380" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="381" spans="1:7">
@@ -8681,13 +8678,13 @@
         <v>4</v>
       </c>
       <c r="C381" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D381" t="s">
         <v>20</v>
       </c>
       <c r="E381" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="382" spans="1:7">
@@ -8698,13 +8695,13 @@
         <v>5</v>
       </c>
       <c r="C382" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D382" t="s">
         <v>21</v>
       </c>
       <c r="E382" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="383" spans="1:7">
@@ -8715,13 +8712,13 @@
         <v>6</v>
       </c>
       <c r="C383" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D383" t="s">
         <v>22</v>
       </c>
       <c r="E383" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="384" spans="1:7">
@@ -8738,7 +8735,7 @@
         <v>23</v>
       </c>
       <c r="E384" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="385" spans="1:7">
@@ -8749,7 +8746,7 @@
         <v>8</v>
       </c>
       <c r="C385" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D385" t="s">
         <v>24</v>
@@ -8760,7 +8757,7 @@
     </row>
     <row r="387" spans="1:7">
       <c r="A387" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="388" spans="1:7">
@@ -8771,10 +8768,10 @@
         <v>35</v>
       </c>
       <c r="D388" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E388" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="E388" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="F388" s="1" t="s">
         <v>38</v>
@@ -8808,7 +8805,7 @@
     </row>
     <row r="390" spans="1:7">
       <c r="A390" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B390">
         <v>0.4</v>
@@ -8923,7 +8920,7 @@
     </row>
     <row r="395" spans="1:7">
       <c r="A395" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B395">
         <v>0.8</v>
@@ -8946,7 +8943,7 @@
     </row>
     <row r="397" spans="1:7">
       <c r="A397" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="398" spans="1:7">
@@ -8988,7 +8985,7 @@
     </row>
     <row r="400" spans="1:7">
       <c r="A400" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B400">
         <v>0</v>
@@ -9068,7 +9065,7 @@
     </row>
     <row r="404" spans="1:6">
       <c r="A404" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B404">
         <v>0</v>
@@ -9108,7 +9105,7 @@
     </row>
     <row r="407" spans="1:6">
       <c r="A407" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="408" spans="1:6">
@@ -9133,7 +9130,7 @@
         <v>1</v>
       </c>
       <c r="C409" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D409" t="s">
         <v>17</v>
@@ -9150,13 +9147,13 @@
         <v>2</v>
       </c>
       <c r="C410" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D410" t="s">
         <v>18</v>
       </c>
       <c r="E410" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="411" spans="1:6">
@@ -9167,13 +9164,13 @@
         <v>3</v>
       </c>
       <c r="C411" t="s">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="D411" t="s">
         <v>19</v>
       </c>
       <c r="E411" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="412" spans="1:6">
@@ -9184,13 +9181,13 @@
         <v>4</v>
       </c>
       <c r="C412" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D412" t="s">
         <v>20</v>
       </c>
       <c r="E412" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="413" spans="1:6">
@@ -9201,13 +9198,13 @@
         <v>5</v>
       </c>
       <c r="C413" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D413" t="s">
         <v>21</v>
       </c>
       <c r="E413" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="414" spans="1:6">
@@ -9218,13 +9215,13 @@
         <v>6</v>
       </c>
       <c r="C414" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D414" t="s">
         <v>22</v>
       </c>
       <c r="E414" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="415" spans="1:6">
@@ -9241,7 +9238,7 @@
         <v>23</v>
       </c>
       <c r="E415" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="416" spans="1:6">
@@ -9252,7 +9249,7 @@
         <v>8</v>
       </c>
       <c r="C416" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D416" t="s">
         <v>24</v>
@@ -9263,7 +9260,7 @@
     </row>
     <row r="418" spans="1:7">
       <c r="A418" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="419" spans="1:7">
@@ -9274,10 +9271,10 @@
         <v>35</v>
       </c>
       <c r="D419" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E419" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="E419" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="F419" s="1" t="s">
         <v>38</v>
@@ -9334,7 +9331,7 @@
     </row>
     <row r="422" spans="1:7">
       <c r="A422" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B422">
         <v>-0.5</v>
@@ -9449,7 +9446,7 @@
     </row>
     <row r="428" spans="1:7">
       <c r="A428" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="429" spans="1:7">
@@ -9491,7 +9488,7 @@
     </row>
     <row r="431" spans="1:7">
       <c r="A431" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B431">
         <v>0</v>
@@ -9611,7 +9608,7 @@
     </row>
     <row r="438" spans="1:6">
       <c r="A438" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="439" spans="1:6">
@@ -9636,7 +9633,7 @@
         <v>1</v>
       </c>
       <c r="C440" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D440" t="s">
         <v>17</v>
@@ -9653,13 +9650,13 @@
         <v>2</v>
       </c>
       <c r="C441" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="D441" t="s">
         <v>18</v>
       </c>
       <c r="E441" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="442" spans="1:6">
@@ -9670,13 +9667,13 @@
         <v>3</v>
       </c>
       <c r="C442" t="s">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="D442" t="s">
         <v>19</v>
       </c>
       <c r="E442" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="443" spans="1:6">
@@ -9687,13 +9684,13 @@
         <v>4</v>
       </c>
       <c r="C443" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="D443" t="s">
         <v>20</v>
       </c>
       <c r="E443" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="444" spans="1:6">
@@ -9704,13 +9701,13 @@
         <v>5</v>
       </c>
       <c r="C444" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D444" t="s">
         <v>21</v>
       </c>
       <c r="E444" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="445" spans="1:6">
@@ -9721,13 +9718,13 @@
         <v>6</v>
       </c>
       <c r="C445" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="D445" t="s">
         <v>22</v>
       </c>
       <c r="E445" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="446" spans="1:6">
@@ -9744,7 +9741,7 @@
         <v>23</v>
       </c>
       <c r="E446" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="447" spans="1:6">
@@ -9755,7 +9752,7 @@
         <v>8</v>
       </c>
       <c r="C447" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D447" t="s">
         <v>24</v>
@@ -9766,7 +9763,7 @@
     </row>
     <row r="449" spans="1:7">
       <c r="A449" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="450" spans="1:7">
@@ -9777,10 +9774,10 @@
         <v>35</v>
       </c>
       <c r="D450" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E450" s="1" t="s">
         <v>131</v>
-      </c>
-      <c r="E450" s="1" t="s">
-        <v>132</v>
       </c>
       <c r="F450" s="1" t="s">
         <v>38</v>
@@ -9883,7 +9880,7 @@
     </row>
     <row r="456" spans="1:7">
       <c r="A456" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="457" spans="1:7">
@@ -9982,7 +9979,7 @@
     </row>
     <row r="463" spans="1:7">
       <c r="A463" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="464" spans="1:7">
@@ -10024,13 +10021,13 @@
         <v>2</v>
       </c>
       <c r="C466" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D466" t="s">
         <v>18</v>
       </c>
       <c r="E466" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="467" spans="1:8">
@@ -10041,13 +10038,13 @@
         <v>3</v>
       </c>
       <c r="C467" t="s">
-        <v>77</v>
+        <v>11</v>
       </c>
       <c r="D467" t="s">
         <v>19</v>
       </c>
       <c r="E467" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="468" spans="1:8">
@@ -10058,13 +10055,13 @@
         <v>4</v>
       </c>
       <c r="C468" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D468" t="s">
         <v>20</v>
       </c>
       <c r="E468" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="469" spans="1:8">
@@ -10075,13 +10072,13 @@
         <v>5</v>
       </c>
       <c r="C469" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D469" t="s">
         <v>21</v>
       </c>
       <c r="E469" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="470" spans="1:8">
@@ -10092,13 +10089,13 @@
         <v>6</v>
       </c>
       <c r="C470" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D470" t="s">
         <v>22</v>
       </c>
       <c r="E470" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="471" spans="1:8">
@@ -10115,7 +10112,7 @@
         <v>23</v>
       </c>
       <c r="E471" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="472" spans="1:8">
@@ -10137,12 +10134,12 @@
     </row>
     <row r="474" spans="1:8">
       <c r="A474" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="475" spans="1:8">
       <c r="B475" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C475" s="1" t="s">
         <v>34</v>
@@ -10269,10 +10266,10 @@
     </row>
     <row r="480" spans="1:8">
       <c r="A480" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B480" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C480">
         <v>-0.1</v>
@@ -10425,10 +10422,10 @@
     </row>
     <row r="486" spans="1:8">
       <c r="A486" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B486" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C486">
         <v>-1.1</v>
@@ -10477,12 +10474,12 @@
     </row>
     <row r="489" spans="1:8">
       <c r="A489" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="490" spans="1:8">
       <c r="B490" s="1" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C490" s="1" t="s">
         <v>34</v>
@@ -10609,10 +10606,10 @@
     </row>
     <row r="495" spans="1:8">
       <c r="A495" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B495" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C495">
         <v>0.4</v>
@@ -10765,10 +10762,10 @@
     </row>
     <row r="501" spans="1:8">
       <c r="A501" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B501" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C501">
         <v>0.3</v>
@@ -10817,12 +10814,12 @@
     </row>
     <row r="504" spans="1:8">
       <c r="A504" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="505" spans="1:8">
       <c r="B505" s="1" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C505" s="1" t="s">
         <v>34</v>
@@ -10949,10 +10946,10 @@
     </row>
     <row r="510" spans="1:8">
       <c r="A510" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B510" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C510">
         <v>0.1</v>
@@ -11105,10 +11102,10 @@
     </row>
     <row r="516" spans="1:8">
       <c r="A516" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B516" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C516">
         <v>0</v>
@@ -11157,12 +11154,12 @@
     </row>
     <row r="519" spans="1:8">
       <c r="A519" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="520" spans="1:8">
       <c r="B520" s="1" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C520" s="1" t="s">
         <v>34</v>
@@ -11289,10 +11286,10 @@
     </row>
     <row r="525" spans="1:8">
       <c r="A525" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B525" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C525">
         <v>0.1</v>
@@ -11445,10 +11442,10 @@
     </row>
     <row r="531" spans="1:8">
       <c r="A531" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B531" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C531">
         <v>0.1</v>
@@ -11497,12 +11494,12 @@
     </row>
     <row r="534" spans="1:8">
       <c r="A534" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="535" spans="1:8">
       <c r="B535" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C535" s="1" t="s">
         <v>34</v>
@@ -11629,10 +11626,10 @@
     </row>
     <row r="540" spans="1:8">
       <c r="A540" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B540" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C540">
         <v>0.3</v>
@@ -11785,10 +11782,10 @@
     </row>
     <row r="546" spans="1:8">
       <c r="A546" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B546" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C546">
         <v>-0.4</v>
@@ -11837,12 +11834,12 @@
     </row>
     <row r="549" spans="1:8">
       <c r="A549" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="550" spans="1:8">
       <c r="B550" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C550" s="1" t="s">
         <v>34</v>
@@ -11969,10 +11966,10 @@
     </row>
     <row r="555" spans="1:8">
       <c r="A555" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B555" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C555">
         <v>-0.6</v>
@@ -12125,10 +12122,10 @@
     </row>
     <row r="561" spans="1:8">
       <c r="A561" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B561" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C561">
         <v>0.6</v>
@@ -12177,7 +12174,7 @@
     </row>
     <row r="564" spans="1:8">
       <c r="A564" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="565" spans="1:8">
@@ -12199,7 +12196,7 @@
     </row>
     <row r="566" spans="1:8">
       <c r="A566" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B566" s="1" t="s">
         <v>40</v>
@@ -12223,7 +12220,7 @@
     <row r="567" spans="1:8">
       <c r="A567" s="1"/>
       <c r="B567" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C567">
         <v>0.1</v>
@@ -12355,7 +12352,7 @@
     <row r="574" spans="1:8">
       <c r="A574" s="1"/>
       <c r="B574" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C574">
         <v>0.5</v>
@@ -12429,7 +12426,7 @@
     </row>
     <row r="578" spans="1:7">
       <c r="A578" s="1" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B578" s="1" t="s">
         <v>40</v>
@@ -12450,7 +12447,7 @@
     <row r="579" spans="1:7">
       <c r="A579" s="1"/>
       <c r="B579" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C579">
         <v>0.5</v>
@@ -12582,7 +12579,7 @@
     <row r="586" spans="1:7">
       <c r="A586" s="1"/>
       <c r="B586" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C586">
         <v>0.1</v>
@@ -12656,7 +12653,7 @@
     </row>
     <row r="590" spans="1:7">
       <c r="A590" s="1" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B590" s="1" t="s">
         <v>40</v>
@@ -12680,7 +12677,7 @@
     <row r="591" spans="1:7">
       <c r="A591" s="1"/>
       <c r="B591" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C591">
         <v>0</v>
@@ -12815,7 +12812,7 @@
     <row r="598" spans="1:7">
       <c r="A598" s="1"/>
       <c r="B598" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C598">
         <v>0.3</v>
@@ -12886,7 +12883,7 @@
     </row>
     <row r="602" spans="1:7">
       <c r="A602" s="1" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B602" s="1" t="s">
         <v>40</v>
@@ -12910,7 +12907,7 @@
     <row r="603" spans="1:7">
       <c r="A603" s="1"/>
       <c r="B603" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C603">
         <v>0.5</v>
@@ -13036,7 +13033,7 @@
     <row r="610" spans="1:7">
       <c r="A610" s="1"/>
       <c r="B610" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C610">
         <v>0.6</v>
@@ -13110,7 +13107,7 @@
     </row>
     <row r="614" spans="1:7">
       <c r="A614" s="1" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B614" s="1" t="s">
         <v>40</v>
@@ -13134,7 +13131,7 @@
     <row r="615" spans="1:7">
       <c r="A615" s="1"/>
       <c r="B615" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C615">
         <v>0</v>
@@ -13269,7 +13266,7 @@
     <row r="622" spans="1:7">
       <c r="A622" s="1"/>
       <c r="B622" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C622">
         <v>0.2</v>
@@ -13346,7 +13343,7 @@
     </row>
     <row r="626" spans="1:7">
       <c r="A626" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B626" s="1" t="s">
         <v>40</v>
@@ -13370,7 +13367,7 @@
     <row r="627" spans="1:7">
       <c r="A627" s="1"/>
       <c r="B627" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C627">
         <v>0.4</v>
@@ -13505,7 +13502,7 @@
     <row r="634" spans="1:7">
       <c r="A634" s="1"/>
       <c r="B634" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C634">
         <v>1</v>

</xml_diff>

<commit_message>
Updated charts so log scales were shown as x-axis ticks instead of gridlines
</commit_message>
<xml_diff>
--- a/assets_output/07_multinomial_logistic_regression.xlsx
+++ b/assets_output/07_multinomial_logistic_regression.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1261" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1261" uniqueCount="186">
   <si>
     <t>MNLogit: 'Entry point into BAHSA services (pathway type and level)', table 0</t>
   </si>
@@ -49,7 +49,7 @@
     <t>y</t>
   </si>
   <si>
-    <t>2026-05-31 15:16</t>
+    <t>2026-06-01 21:48</t>
   </si>
   <si>
     <t>3391</t>
@@ -245,6 +245,9 @@
   </si>
   <si>
     <t>rt_outcome</t>
+  </si>
+  <si>
+    <t>2026-06-01 21:49</t>
   </si>
   <si>
     <t>2195</t>
@@ -5371,7 +5374,7 @@
         <v>18</v>
       </c>
       <c r="E213" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="214" spans="1:8">
@@ -5382,13 +5385,13 @@
         <v>3</v>
       </c>
       <c r="C214" t="s">
-        <v>11</v>
+        <v>77</v>
       </c>
       <c r="D214" t="s">
         <v>19</v>
       </c>
       <c r="E214" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="215" spans="1:8">
@@ -5399,13 +5402,13 @@
         <v>4</v>
       </c>
       <c r="C215" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D215" t="s">
         <v>20</v>
       </c>
       <c r="E215" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="216" spans="1:8">
@@ -5416,13 +5419,13 @@
         <v>5</v>
       </c>
       <c r="C216" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D216" t="s">
         <v>21</v>
       </c>
       <c r="E216" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="217" spans="1:8">
@@ -5433,13 +5436,13 @@
         <v>6</v>
       </c>
       <c r="C217" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D217" t="s">
         <v>22</v>
       </c>
       <c r="E217" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="218" spans="1:8">
@@ -5456,7 +5459,7 @@
         <v>23</v>
       </c>
       <c r="E218" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="219" spans="1:8">
@@ -5467,7 +5470,7 @@
         <v>8</v>
       </c>
       <c r="C219" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D219" t="s">
         <v>24</v>
@@ -5478,12 +5481,12 @@
     </row>
     <row r="221" spans="1:8">
       <c r="A221" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="222" spans="1:8">
       <c r="B222" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C222" s="1" t="s">
         <v>34</v>
@@ -5610,10 +5613,10 @@
     </row>
     <row r="227" spans="1:8">
       <c r="A227" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B227" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C227">
         <v>0.3</v>
@@ -5740,10 +5743,10 @@
     </row>
     <row r="232" spans="1:8">
       <c r="A232" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B232" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C232">
         <v>1.7</v>
@@ -5792,12 +5795,12 @@
     </row>
     <row r="235" spans="1:8">
       <c r="A235" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="236" spans="1:8">
       <c r="B236" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C236" s="1" t="s">
         <v>34</v>
@@ -5924,10 +5927,10 @@
     </row>
     <row r="241" spans="1:8">
       <c r="A241" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B241" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C241">
         <v>0.1</v>
@@ -6054,10 +6057,10 @@
     </row>
     <row r="246" spans="1:8">
       <c r="A246" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B246" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C246">
         <v>2</v>
@@ -6106,12 +6109,12 @@
     </row>
     <row r="249" spans="1:8">
       <c r="A249" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="250" spans="1:8">
       <c r="B250" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C250" s="1" t="s">
         <v>34</v>
@@ -6238,10 +6241,10 @@
     </row>
     <row r="255" spans="1:8">
       <c r="A255" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B255" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C255">
         <v>-0.5</v>
@@ -6368,10 +6371,10 @@
     </row>
     <row r="260" spans="1:8">
       <c r="A260" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B260" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C260">
         <v>2.9</v>
@@ -6420,7 +6423,7 @@
     </row>
     <row r="263" spans="1:8">
       <c r="A263" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="264" spans="1:8">
@@ -6442,7 +6445,7 @@
     </row>
     <row r="265" spans="1:8">
       <c r="A265" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B265" s="1" t="s">
         <v>40</v>
@@ -6466,7 +6469,7 @@
     <row r="266" spans="1:8">
       <c r="A266" s="1"/>
       <c r="B266" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C266">
         <v>0.3</v>
@@ -6574,7 +6577,7 @@
     <row r="272" spans="1:8">
       <c r="A272" s="1"/>
       <c r="B272" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C272">
         <v>0</v>
@@ -6651,7 +6654,7 @@
     </row>
     <row r="276" spans="1:7">
       <c r="A276" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B276" s="1" t="s">
         <v>40</v>
@@ -6675,7 +6678,7 @@
     <row r="277" spans="1:7">
       <c r="A277" s="1"/>
       <c r="B277" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C277">
         <v>0</v>
@@ -6798,7 +6801,7 @@
     <row r="283" spans="1:7">
       <c r="A283" s="1"/>
       <c r="B283" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C283">
         <v>0</v>
@@ -6878,7 +6881,7 @@
     </row>
     <row r="287" spans="1:7">
       <c r="A287" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B287" s="1" t="s">
         <v>40</v>
@@ -6902,7 +6905,7 @@
     <row r="288" spans="1:7">
       <c r="A288" s="1"/>
       <c r="B288" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C288">
         <v>0.3</v>
@@ -7019,7 +7022,7 @@
     <row r="294" spans="1:7">
       <c r="A294" s="1"/>
       <c r="B294" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C294">
         <v>0</v>
@@ -7099,7 +7102,7 @@
     </row>
     <row r="299" spans="1:7">
       <c r="A299" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="300" spans="1:7">
@@ -7141,13 +7144,13 @@
         <v>2</v>
       </c>
       <c r="C302" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D302" t="s">
         <v>18</v>
       </c>
       <c r="E302" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="303" spans="1:7">
@@ -7158,13 +7161,13 @@
         <v>3</v>
       </c>
       <c r="C303" t="s">
-        <v>11</v>
+        <v>77</v>
       </c>
       <c r="D303" t="s">
         <v>19</v>
       </c>
       <c r="E303" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="304" spans="1:7">
@@ -7175,13 +7178,13 @@
         <v>4</v>
       </c>
       <c r="C304" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D304" t="s">
         <v>20</v>
       </c>
       <c r="E304" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="305" spans="1:8">
@@ -7192,13 +7195,13 @@
         <v>5</v>
       </c>
       <c r="C305" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D305" t="s">
         <v>21</v>
       </c>
       <c r="E305" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="306" spans="1:8">
@@ -7209,13 +7212,13 @@
         <v>6</v>
       </c>
       <c r="C306" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D306" t="s">
         <v>22</v>
       </c>
       <c r="E306" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="307" spans="1:8">
@@ -7232,7 +7235,7 @@
         <v>23</v>
       </c>
       <c r="E307" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="308" spans="1:8">
@@ -7243,7 +7246,7 @@
         <v>8</v>
       </c>
       <c r="C308" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D308" t="s">
         <v>24</v>
@@ -7254,12 +7257,12 @@
     </row>
     <row r="310" spans="1:8">
       <c r="A310" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
     </row>
     <row r="311" spans="1:8">
       <c r="B311" s="1" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C311" s="1" t="s">
         <v>34</v>
@@ -7360,10 +7363,10 @@
     </row>
     <row r="315" spans="1:8">
       <c r="A315" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B315" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C315">
         <v>0.3</v>
@@ -7490,10 +7493,10 @@
     </row>
     <row r="320" spans="1:8">
       <c r="A320" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B320" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C320">
         <v>1.7</v>
@@ -7516,12 +7519,12 @@
     </row>
     <row r="322" spans="1:8">
       <c r="A322" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="323" spans="1:8">
       <c r="B323" s="1" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C323" s="1" t="s">
         <v>34</v>
@@ -7622,10 +7625,10 @@
     </row>
     <row r="327" spans="1:8">
       <c r="A327" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B327" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C327">
         <v>0.2</v>
@@ -7752,10 +7755,10 @@
     </row>
     <row r="332" spans="1:8">
       <c r="A332" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B332" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C332">
         <v>1.8</v>
@@ -7778,12 +7781,12 @@
     </row>
     <row r="334" spans="1:8">
       <c r="A334" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
     </row>
     <row r="335" spans="1:8">
       <c r="B335" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C335" s="1" t="s">
         <v>34</v>
@@ -7884,10 +7887,10 @@
     </row>
     <row r="339" spans="1:8">
       <c r="A339" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B339" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C339">
         <v>-0.5</v>
@@ -8014,10 +8017,10 @@
     </row>
     <row r="344" spans="1:8">
       <c r="A344" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B344" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C344">
         <v>2.2</v>
@@ -8040,7 +8043,7 @@
     </row>
     <row r="346" spans="1:8">
       <c r="A346" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="347" spans="1:8">
@@ -8062,7 +8065,7 @@
     </row>
     <row r="348" spans="1:8">
       <c r="A348" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B348" s="1" t="s">
         <v>40</v>
@@ -8086,7 +8089,7 @@
     <row r="349" spans="1:8">
       <c r="A349" s="1"/>
       <c r="B349" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C349">
         <v>0.3</v>
@@ -8158,7 +8161,7 @@
     <row r="353" spans="1:7">
       <c r="A353" s="1"/>
       <c r="B353" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C353">
         <v>0.1</v>
@@ -8232,7 +8235,7 @@
     </row>
     <row r="357" spans="1:7">
       <c r="A357" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B357" s="1" t="s">
         <v>40</v>
@@ -8256,7 +8259,7 @@
     <row r="358" spans="1:7">
       <c r="A358" s="1"/>
       <c r="B358" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C358">
         <v>0</v>
@@ -8340,7 +8343,7 @@
     <row r="362" spans="1:7">
       <c r="A362" s="1"/>
       <c r="B362" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C362">
         <v>0</v>
@@ -8420,7 +8423,7 @@
     </row>
     <row r="366" spans="1:7">
       <c r="A366" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B366" s="1" t="s">
         <v>40</v>
@@ -8444,7 +8447,7 @@
     <row r="367" spans="1:7">
       <c r="A367" s="1"/>
       <c r="B367" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C367">
         <v>0.1</v>
@@ -8522,7 +8525,7 @@
     <row r="371" spans="1:7">
       <c r="A371" s="1"/>
       <c r="B371" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C371">
         <v>0</v>
@@ -8602,7 +8605,7 @@
     </row>
     <row r="376" spans="1:7">
       <c r="A376" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="377" spans="1:7">
@@ -8627,7 +8630,7 @@
         <v>1</v>
       </c>
       <c r="C378" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D378" t="s">
         <v>17</v>
@@ -8644,13 +8647,13 @@
         <v>2</v>
       </c>
       <c r="C379" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D379" t="s">
         <v>18</v>
       </c>
       <c r="E379" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="380" spans="1:7">
@@ -8661,13 +8664,13 @@
         <v>3</v>
       </c>
       <c r="C380" t="s">
-        <v>11</v>
+        <v>77</v>
       </c>
       <c r="D380" t="s">
         <v>19</v>
       </c>
       <c r="E380" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="381" spans="1:7">
@@ -8678,13 +8681,13 @@
         <v>4</v>
       </c>
       <c r="C381" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D381" t="s">
         <v>20</v>
       </c>
       <c r="E381" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="382" spans="1:7">
@@ -8695,13 +8698,13 @@
         <v>5</v>
       </c>
       <c r="C382" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D382" t="s">
         <v>21</v>
       </c>
       <c r="E382" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="383" spans="1:7">
@@ -8712,13 +8715,13 @@
         <v>6</v>
       </c>
       <c r="C383" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D383" t="s">
         <v>22</v>
       </c>
       <c r="E383" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="384" spans="1:7">
@@ -8735,7 +8738,7 @@
         <v>23</v>
       </c>
       <c r="E384" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="385" spans="1:7">
@@ -8746,7 +8749,7 @@
         <v>8</v>
       </c>
       <c r="C385" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D385" t="s">
         <v>24</v>
@@ -8757,7 +8760,7 @@
     </row>
     <row r="387" spans="1:7">
       <c r="A387" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="388" spans="1:7">
@@ -8768,10 +8771,10 @@
         <v>35</v>
       </c>
       <c r="D388" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E388" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F388" s="1" t="s">
         <v>38</v>
@@ -8805,7 +8808,7 @@
     </row>
     <row r="390" spans="1:7">
       <c r="A390" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B390">
         <v>0.4</v>
@@ -8920,7 +8923,7 @@
     </row>
     <row r="395" spans="1:7">
       <c r="A395" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B395">
         <v>0.8</v>
@@ -8943,7 +8946,7 @@
     </row>
     <row r="397" spans="1:7">
       <c r="A397" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="398" spans="1:7">
@@ -8985,7 +8988,7 @@
     </row>
     <row r="400" spans="1:7">
       <c r="A400" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B400">
         <v>0</v>
@@ -9065,7 +9068,7 @@
     </row>
     <row r="404" spans="1:6">
       <c r="A404" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B404">
         <v>0</v>
@@ -9105,7 +9108,7 @@
     </row>
     <row r="407" spans="1:6">
       <c r="A407" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="408" spans="1:6">
@@ -9130,7 +9133,7 @@
         <v>1</v>
       </c>
       <c r="C409" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D409" t="s">
         <v>17</v>
@@ -9147,13 +9150,13 @@
         <v>2</v>
       </c>
       <c r="C410" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D410" t="s">
         <v>18</v>
       </c>
       <c r="E410" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="411" spans="1:6">
@@ -9164,13 +9167,13 @@
         <v>3</v>
       </c>
       <c r="C411" t="s">
-        <v>11</v>
+        <v>77</v>
       </c>
       <c r="D411" t="s">
         <v>19</v>
       </c>
       <c r="E411" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="412" spans="1:6">
@@ -9181,13 +9184,13 @@
         <v>4</v>
       </c>
       <c r="C412" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D412" t="s">
         <v>20</v>
       </c>
       <c r="E412" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="413" spans="1:6">
@@ -9198,13 +9201,13 @@
         <v>5</v>
       </c>
       <c r="C413" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="D413" t="s">
         <v>21</v>
       </c>
       <c r="E413" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="414" spans="1:6">
@@ -9215,13 +9218,13 @@
         <v>6</v>
       </c>
       <c r="C414" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D414" t="s">
         <v>22</v>
       </c>
       <c r="E414" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="415" spans="1:6">
@@ -9238,7 +9241,7 @@
         <v>23</v>
       </c>
       <c r="E415" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="416" spans="1:6">
@@ -9249,7 +9252,7 @@
         <v>8</v>
       </c>
       <c r="C416" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="D416" t="s">
         <v>24</v>
@@ -9260,7 +9263,7 @@
     </row>
     <row r="418" spans="1:7">
       <c r="A418" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="419" spans="1:7">
@@ -9271,10 +9274,10 @@
         <v>35</v>
       </c>
       <c r="D419" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E419" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F419" s="1" t="s">
         <v>38</v>
@@ -9331,7 +9334,7 @@
     </row>
     <row r="422" spans="1:7">
       <c r="A422" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B422">
         <v>-0.5</v>
@@ -9446,7 +9449,7 @@
     </row>
     <row r="428" spans="1:7">
       <c r="A428" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="429" spans="1:7">
@@ -9488,7 +9491,7 @@
     </row>
     <row r="431" spans="1:7">
       <c r="A431" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B431">
         <v>0</v>
@@ -9608,7 +9611,7 @@
     </row>
     <row r="438" spans="1:6">
       <c r="A438" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="439" spans="1:6">
@@ -9633,7 +9636,7 @@
         <v>1</v>
       </c>
       <c r="C440" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D440" t="s">
         <v>17</v>
@@ -9650,13 +9653,13 @@
         <v>2</v>
       </c>
       <c r="C441" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="D441" t="s">
         <v>18</v>
       </c>
       <c r="E441" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="442" spans="1:6">
@@ -9667,13 +9670,13 @@
         <v>3</v>
       </c>
       <c r="C442" t="s">
-        <v>11</v>
+        <v>77</v>
       </c>
       <c r="D442" t="s">
         <v>19</v>
       </c>
       <c r="E442" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="443" spans="1:6">
@@ -9684,13 +9687,13 @@
         <v>4</v>
       </c>
       <c r="C443" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D443" t="s">
         <v>20</v>
       </c>
       <c r="E443" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
     </row>
     <row r="444" spans="1:6">
@@ -9701,13 +9704,13 @@
         <v>5</v>
       </c>
       <c r="C444" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="D444" t="s">
         <v>21</v>
       </c>
       <c r="E444" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="445" spans="1:6">
@@ -9718,13 +9721,13 @@
         <v>6</v>
       </c>
       <c r="C445" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D445" t="s">
         <v>22</v>
       </c>
       <c r="E445" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="446" spans="1:6">
@@ -9741,7 +9744,7 @@
         <v>23</v>
       </c>
       <c r="E446" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="447" spans="1:6">
@@ -9752,7 +9755,7 @@
         <v>8</v>
       </c>
       <c r="C447" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D447" t="s">
         <v>24</v>
@@ -9763,7 +9766,7 @@
     </row>
     <row r="449" spans="1:7">
       <c r="A449" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="450" spans="1:7">
@@ -9774,10 +9777,10 @@
         <v>35</v>
       </c>
       <c r="D450" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E450" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F450" s="1" t="s">
         <v>38</v>
@@ -9880,7 +9883,7 @@
     </row>
     <row r="456" spans="1:7">
       <c r="A456" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="457" spans="1:7">
@@ -9979,7 +9982,7 @@
     </row>
     <row r="463" spans="1:7">
       <c r="A463" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="464" spans="1:7">
@@ -10021,13 +10024,13 @@
         <v>2</v>
       </c>
       <c r="C466" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D466" t="s">
         <v>18</v>
       </c>
       <c r="E466" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="467" spans="1:8">
@@ -10038,13 +10041,13 @@
         <v>3</v>
       </c>
       <c r="C467" t="s">
-        <v>11</v>
+        <v>77</v>
       </c>
       <c r="D467" t="s">
         <v>19</v>
       </c>
       <c r="E467" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="468" spans="1:8">
@@ -10055,13 +10058,13 @@
         <v>4</v>
       </c>
       <c r="C468" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D468" t="s">
         <v>20</v>
       </c>
       <c r="E468" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="469" spans="1:8">
@@ -10072,13 +10075,13 @@
         <v>5</v>
       </c>
       <c r="C469" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D469" t="s">
         <v>21</v>
       </c>
       <c r="E469" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="470" spans="1:8">
@@ -10089,13 +10092,13 @@
         <v>6</v>
       </c>
       <c r="C470" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D470" t="s">
         <v>22</v>
       </c>
       <c r="E470" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="471" spans="1:8">
@@ -10112,7 +10115,7 @@
         <v>23</v>
       </c>
       <c r="E471" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="472" spans="1:8">
@@ -10134,12 +10137,12 @@
     </row>
     <row r="474" spans="1:8">
       <c r="A474" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
     </row>
     <row r="475" spans="1:8">
       <c r="B475" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C475" s="1" t="s">
         <v>34</v>
@@ -10266,10 +10269,10 @@
     </row>
     <row r="480" spans="1:8">
       <c r="A480" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B480" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C480">
         <v>-0.1</v>
@@ -10422,10 +10425,10 @@
     </row>
     <row r="486" spans="1:8">
       <c r="A486" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B486" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C486">
         <v>-1.1</v>
@@ -10474,12 +10477,12 @@
     </row>
     <row r="489" spans="1:8">
       <c r="A489" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="490" spans="1:8">
       <c r="B490" s="1" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C490" s="1" t="s">
         <v>34</v>
@@ -10606,10 +10609,10 @@
     </row>
     <row r="495" spans="1:8">
       <c r="A495" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B495" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C495">
         <v>0.4</v>
@@ -10762,10 +10765,10 @@
     </row>
     <row r="501" spans="1:8">
       <c r="A501" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B501" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C501">
         <v>0.3</v>
@@ -10814,12 +10817,12 @@
     </row>
     <row r="504" spans="1:8">
       <c r="A504" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
     </row>
     <row r="505" spans="1:8">
       <c r="B505" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C505" s="1" t="s">
         <v>34</v>
@@ -10946,10 +10949,10 @@
     </row>
     <row r="510" spans="1:8">
       <c r="A510" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B510" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C510">
         <v>0.1</v>
@@ -11102,10 +11105,10 @@
     </row>
     <row r="516" spans="1:8">
       <c r="A516" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B516" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C516">
         <v>0</v>
@@ -11154,12 +11157,12 @@
     </row>
     <row r="519" spans="1:8">
       <c r="A519" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
     </row>
     <row r="520" spans="1:8">
       <c r="B520" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C520" s="1" t="s">
         <v>34</v>
@@ -11286,10 +11289,10 @@
     </row>
     <row r="525" spans="1:8">
       <c r="A525" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B525" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C525">
         <v>0.1</v>
@@ -11442,10 +11445,10 @@
     </row>
     <row r="531" spans="1:8">
       <c r="A531" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B531" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C531">
         <v>0.1</v>
@@ -11494,12 +11497,12 @@
     </row>
     <row r="534" spans="1:8">
       <c r="A534" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="535" spans="1:8">
       <c r="B535" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C535" s="1" t="s">
         <v>34</v>
@@ -11626,10 +11629,10 @@
     </row>
     <row r="540" spans="1:8">
       <c r="A540" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B540" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C540">
         <v>0.3</v>
@@ -11782,10 +11785,10 @@
     </row>
     <row r="546" spans="1:8">
       <c r="A546" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B546" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C546">
         <v>-0.4</v>
@@ -11834,12 +11837,12 @@
     </row>
     <row r="549" spans="1:8">
       <c r="A549" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="550" spans="1:8">
       <c r="B550" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C550" s="1" t="s">
         <v>34</v>
@@ -11966,10 +11969,10 @@
     </row>
     <row r="555" spans="1:8">
       <c r="A555" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B555" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C555">
         <v>-0.6</v>
@@ -12122,10 +12125,10 @@
     </row>
     <row r="561" spans="1:8">
       <c r="A561" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B561" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C561">
         <v>0.6</v>
@@ -12174,7 +12177,7 @@
     </row>
     <row r="564" spans="1:8">
       <c r="A564" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="565" spans="1:8">
@@ -12196,7 +12199,7 @@
     </row>
     <row r="566" spans="1:8">
       <c r="A566" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B566" s="1" t="s">
         <v>40</v>
@@ -12220,7 +12223,7 @@
     <row r="567" spans="1:8">
       <c r="A567" s="1"/>
       <c r="B567" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C567">
         <v>0.1</v>
@@ -12352,7 +12355,7 @@
     <row r="574" spans="1:8">
       <c r="A574" s="1"/>
       <c r="B574" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C574">
         <v>0.5</v>
@@ -12426,7 +12429,7 @@
     </row>
     <row r="578" spans="1:7">
       <c r="A578" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B578" s="1" t="s">
         <v>40</v>
@@ -12447,7 +12450,7 @@
     <row r="579" spans="1:7">
       <c r="A579" s="1"/>
       <c r="B579" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C579">
         <v>0.5</v>
@@ -12579,7 +12582,7 @@
     <row r="586" spans="1:7">
       <c r="A586" s="1"/>
       <c r="B586" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C586">
         <v>0.1</v>
@@ -12653,7 +12656,7 @@
     </row>
     <row r="590" spans="1:7">
       <c r="A590" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B590" s="1" t="s">
         <v>40</v>
@@ -12677,7 +12680,7 @@
     <row r="591" spans="1:7">
       <c r="A591" s="1"/>
       <c r="B591" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C591">
         <v>0</v>
@@ -12812,7 +12815,7 @@
     <row r="598" spans="1:7">
       <c r="A598" s="1"/>
       <c r="B598" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C598">
         <v>0.3</v>
@@ -12883,7 +12886,7 @@
     </row>
     <row r="602" spans="1:7">
       <c r="A602" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B602" s="1" t="s">
         <v>40</v>
@@ -12907,7 +12910,7 @@
     <row r="603" spans="1:7">
       <c r="A603" s="1"/>
       <c r="B603" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C603">
         <v>0.5</v>
@@ -13033,7 +13036,7 @@
     <row r="610" spans="1:7">
       <c r="A610" s="1"/>
       <c r="B610" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C610">
         <v>0.6</v>
@@ -13107,7 +13110,7 @@
     </row>
     <row r="614" spans="1:7">
       <c r="A614" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B614" s="1" t="s">
         <v>40</v>
@@ -13131,7 +13134,7 @@
     <row r="615" spans="1:7">
       <c r="A615" s="1"/>
       <c r="B615" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C615">
         <v>0</v>
@@ -13266,7 +13269,7 @@
     <row r="622" spans="1:7">
       <c r="A622" s="1"/>
       <c r="B622" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C622">
         <v>0.2</v>
@@ -13343,7 +13346,7 @@
     </row>
     <row r="626" spans="1:7">
       <c r="A626" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B626" s="1" t="s">
         <v>40</v>
@@ -13367,7 +13370,7 @@
     <row r="627" spans="1:7">
       <c r="A627" s="1"/>
       <c r="B627" s="1" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C627">
         <v>0.4</v>
@@ -13502,7 +13505,7 @@
     <row r="634" spans="1:7">
       <c r="A634" s="1"/>
       <c r="B634" s="1" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C634">
         <v>1</v>

</xml_diff>